<commit_message>
Build connector-ready executive briefing pipeline
</commit_message>
<xml_diff>
--- a/outputs/executive-briefing-machine-demo/executive-briefing-demo.xlsx
+++ b/outputs/executive-briefing-machine-demo/executive-briefing-demo.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R8d4baa0d255d4ead"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="Re263f07d90ba41ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="3" r:id="R383a30c4cc96469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R1237e7480f064a15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="R99baa06ef0cf481b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="3" r:id="Raa8ee6bee0f543fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -228,7 +228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4817ed9ee8084453"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R752b71a91d1d4d13"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -466,10 +466,10 @@
         <x:v>-5k vs last month</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>Self-serve analytics export shipped to general availability after the final rollout guardrails cleared.</x:v>
+        <x:v>Support backlog dropped below 24 hours for the first time in six weeks after the triage rotation change.</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>The mobile crash regression fix is still waiting on final QA signoff.</x:v>
+        <x:v>Finance flagged June vendor spend as slightly ahead of plan because of the analytics infrastructure migration.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -716,7 +716,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R160eb7e0fc094331"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b36bed25d0d49bc"/>
 </x:worksheet>
 </file>
 
@@ -725,7 +725,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="140" customWidth="1"/>
-    <x:col min="2" max="2" width="120" customWidth="1"/>
+    <x:col min="2" max="2" width="160" customWidth="1"/>
     <x:col min="3" max="3" width="255" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -770,7 +770,7 @@
         <x:v>Highlight</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Self-serve analytics export shipped to general availability after the final rollout guardrails cleared.</x:v>
+        <x:v>Support backlog dropped below 24 hours for the first time in six weeks after the triage rotation change.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -803,7 +803,7 @@
         <x:v>Risk</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>The mobile crash regression fix is still waiting on final QA signoff.</x:v>
+        <x:v>Finance flagged June vendor spend as slightly ahead of plan because of the analytics infrastructure migration.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -848,6 +848,61 @@
       </x:c>
       <x:c r="C11" t="str">
         <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>slack</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Slack-ready connector contract</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>github</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>GitHub-ready connector contract</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>local-notes</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Local document ingestion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>kpi-file</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Spreadsheet/file ingestion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>computer-use</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>stubbed</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>computer-use for UI-only dashboards and internal tools</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add live Slack adapter and scheduled briefing runner
</commit_message>
<xml_diff>
--- a/outputs/executive-briefing-machine-demo/executive-briefing-demo.xlsx
+++ b/outputs/executive-briefing-machine-demo/executive-briefing-demo.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R1237e7480f064a15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="R99baa06ef0cf481b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="3" r:id="Raa8ee6bee0f543fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rf78fc519c4f24aef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="R21feaf78a59743a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="3" r:id="R4392da7c62804f02"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -228,7 +228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R752b71a91d1d4d13"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0fa2367908b348b5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -716,7 +716,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b36bed25d0d49bc"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0503781459e54bc2"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Tighten live Slack filtering for executive briefing
</commit_message>
<xml_diff>
--- a/outputs/executive-briefing-machine-demo/executive-briefing-demo.xlsx
+++ b/outputs/executive-briefing-machine-demo/executive-briefing-demo.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rf78fc519c4f24aef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="R21feaf78a59743a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="3" r:id="R4392da7c62804f02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Ra8ef93d911b44400"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="R2602f5b148e14458"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="3" r:id="R31a3af841b144c6f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -228,7 +228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0fa2367908b348b5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2ae82c98a9a245a3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -432,11 +432,9 @@
         <x:v>+64k vs last month</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>Growth team rolled out the onboarding checklist experiment to 40% of new workspaces and activation improved by 6 percentage points in the pilot group.</x:v>
-      </x:c>
-      <x:c r="F5" t="str">
-        <x:v>Two enterprise deals are blocked on security questionnaire turnaround and legal review.</x:v>
-      </x:c>
+        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
+      </x:c>
+      <x:c r="F5" t="str"/>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" t="str">
@@ -449,11 +447,9 @@
         <x:v>+85k vs last month</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>Northstar expanded to an annual plan, adding $48k ARR after the joint sales and success push closed this week.</x:v>
-      </x:c>
-      <x:c r="F6" t="str">
-        <x:v>The iOS 3.12 release introduced a crash regression affecting 4.7% of mobile sessions.</x:v>
-      </x:c>
+        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
+      </x:c>
+      <x:c r="F6" t="str"/>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" t="str">
@@ -466,11 +462,9 @@
         <x:v>-5k vs last month</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>Support backlog dropped below 24 hours for the first time in six weeks after the triage rotation change.</x:v>
-      </x:c>
-      <x:c r="F7" t="str">
-        <x:v>Finance flagged June vendor spend as slightly ahead of plan because of the analytics infrastructure migration.</x:v>
-      </x:c>
+        <x:v>Make the narrative concrete: growth is working, but reliability and enterprise readiness still need disciplined execution.</x:v>
+      </x:c>
+      <x:c r="F7" t="str"/>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" t="str">
@@ -507,7 +501,7 @@
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" t="str">
-        <x:v>Approve short-term legal support for enterprise security reviews.</x:v>
+        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
       </x:c>
       <x:c r="B12" t="str">
         <x:v>CEO / Legal</x:v>
@@ -518,7 +512,7 @@
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
       <x:c r="A13" t="str">
-        <x:v>Prioritize the mobile crash hotfix ahead of lower-priority roadmap work.</x:v>
+        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
       </x:c>
       <x:c r="B13" t="str">
         <x:v>Product / Engineering</x:v>
@@ -528,9 +522,7 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
-      <x:c r="A14" t="str">
-        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
-      </x:c>
+      <x:c r="A14" t="str"/>
       <x:c r="B14" t="str">
         <x:v>Leadership team</x:v>
       </x:c>
@@ -539,9 +531,7 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="38" customHeight="1">
-      <x:c r="A15" t="str">
-        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
-      </x:c>
+      <x:c r="A15" t="str"/>
       <x:c r="B15" t="str">
         <x:v>Exec staff</x:v>
       </x:c>
@@ -716,7 +706,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0503781459e54bc2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaf33a20550247dd"/>
 </x:worksheet>
 </file>
 
@@ -748,7 +738,7 @@
         <x:v>Highlight</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Growth team rolled out the onboarding checklist experiment to 40% of new workspaces and activation improved by 6 percentage points in the pilot group.</x:v>
+        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -759,7 +749,7 @@
         <x:v>Highlight</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Northstar expanded to an annual plan, adding $48k ARR after the joint sales and success push closed this week.</x:v>
+        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -770,138 +760,83 @@
         <x:v>Highlight</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Support backlog dropped below 24 hours for the first time in six weeks after the triage rotation change.</x:v>
+        <x:v>Make the narrative concrete: growth is working, but reliability and enterprise readiness still need disciplined execution.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Slack/GitHub</x:v>
+        <x:v>Leadership/Slack</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Risk</x:v>
+        <x:v>Ask</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Two enterprise deals are blocked on security questionnaire turnaround and legal review.</x:v>
+        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Slack/GitHub</x:v>
+        <x:v>Leadership/Slack</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Risk</x:v>
+        <x:v>Ask</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>The iOS 3.12 release introduced a crash regression affecting 4.7% of mobile sessions.</x:v>
+        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Slack/GitHub</x:v>
+        <x:v>slack</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Risk</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Finance flagged June vendor spend as slightly ahead of plan because of the analytics infrastructure migration.</x:v>
+        <x:v>Live Slack API adapter for 2 channel(s)</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Leadership/Slack</x:v>
+        <x:v>github</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Ask</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>Approve short-term legal support for enterprise security reviews.</x:v>
+        <x:v>Live GitHub API adapter for Laksh-star/codex-workflow-agents</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Leadership/Slack</x:v>
+        <x:v>local-notes</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>Ask</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>Prioritize the mobile crash hotfix ahead of lower-priority roadmap work.</x:v>
+        <x:v>Local document ingestion</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Leadership/Slack</x:v>
+        <x:v>kpi-file</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>Ask</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
+        <x:v>Spreadsheet/file ingestion</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>Leadership/Slack</x:v>
+        <x:v>computer-use</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Ask</x:v>
+        <x:v>stubbed</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>slack</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:v>implemented</x:v>
-      </x:c>
-      <x:c r="C12" t="str">
-        <x:v>Slack-ready connector contract</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>github</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>implemented</x:v>
-      </x:c>
-      <x:c r="C13" t="str">
-        <x:v>GitHub-ready connector contract</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>local-notes</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>implemented</x:v>
-      </x:c>
-      <x:c r="C14" t="str">
-        <x:v>Local document ingestion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>kpi-file</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>implemented</x:v>
-      </x:c>
-      <x:c r="C15" t="str">
-        <x:v>Spreadsheet/file ingestion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>computer-use</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>stubbed</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
         <x:v>computer-use for UI-only dashboards and internal tools</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Tune Slack classifier for consulting signals
</commit_message>
<xml_diff>
--- a/outputs/executive-briefing-machine-demo/executive-briefing-demo.xlsx
+++ b/outputs/executive-briefing-machine-demo/executive-briefing-demo.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Ra8ef93d911b44400"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="R2602f5b148e14458"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="3" r:id="R31a3af841b144c6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R611cf8399d664131"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="R52320bc482874aad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="3" r:id="R884a9bf76a484d8e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -228,7 +228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2ae82c98a9a245a3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R16ff1b2fdd0944b9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -432,9 +432,11 @@
         <x:v>+64k vs last month</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
-      </x:c>
-      <x:c r="F5" t="str"/>
+        <x:v>C09MXSVB2HH: • The CEO of the retail client said the weekly advisory cadence is working, but they want tighter decision logs and clearer owner follow-through. • The operations lead asked for a dashboard pack that shows burn, renewal risk, and implementation blockers in one place. • This is a good expansion signal if we package the reporting layer cleanly.</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>C09MXSVB2HH: • One client workshop is blocked until the data room access issue is resolved. • Delivery confidence remains high, but the team needs a named owner for exec stakeholder scheduling. • If we do not unblock the security questionnaire by Friday, the healthcare advisory kickoff will slip by at least one week.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" t="str">
@@ -447,9 +449,11 @@
         <x:v>+85k vs last month</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
-      </x:c>
-      <x:c r="F6" t="str"/>
+        <x:v>C09MXSVB2HH: • Qualified consulting pipeline moved from _$118k to $164k_ over the last 10 days. • Two enterprise advisory opportunities are now in procurement review. • The near-term risk is slower legal turnaround on MSA redlines, which could push one April close into May.</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>Open issue #5: Risk: Live channel quality can overwhelm executive-briefing signal</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" t="str">
@@ -462,9 +466,11 @@
         <x:v>-5k vs last month</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>Make the narrative concrete: growth is working, but reliability and enterprise readiness still need disciplined execution.</x:v>
-      </x:c>
-      <x:c r="F7" t="str"/>
+        <x:v>C09MXSVB2HH: Hyperagent is a good alternative for clients, in advanced talks with RTPL for its implementaiotn on behalf of DB consulting and Advisory</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Open issue #4: Future idea: Add client-ready QBR output mode</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" t="str">
@@ -501,7 +507,7 @@
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
       <x:c r="A12" t="str">
-        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
+        <x:v>C09MXSVB2HH: • Need approval to pull one additional analytics contractor into the customer-ops workstream for 3 weeks. • Need legal support on the enterprise MSA backlog to protect April revenue timing. • Please confirm whether we want the board narrative to emphasize pipeline quality, delivery readiness, or margin improvement first.</x:v>
       </x:c>
       <x:c r="B12" t="str">
         <x:v>CEO / Legal</x:v>
@@ -512,7 +518,7 @@
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
       <x:c r="A13" t="str">
-        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
+        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
       </x:c>
       <x:c r="B13" t="str">
         <x:v>Product / Engineering</x:v>
@@ -522,7 +528,9 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
-      <x:c r="A14" t="str"/>
+      <x:c r="A14" t="str">
+        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
+      </x:c>
       <x:c r="B14" t="str">
         <x:v>Leadership team</x:v>
       </x:c>
@@ -706,7 +714,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaf33a20550247dd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56fbe2dad6b6428e"/>
 </x:worksheet>
 </file>
 
@@ -738,7 +746,7 @@
         <x:v>Highlight</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
+        <x:v>C09MXSVB2HH: • The CEO of the retail client said the weekly advisory cadence is working, but they want tighter decision logs and clearer owner follow-through. • The operations lead asked for a dashboard pack that shows burn, renewal risk, and implementation blockers in one place. • This is a good expansion signal if we package the reporting layer cleanly.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -749,7 +757,7 @@
         <x:v>Highlight</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
+        <x:v>C09MXSVB2HH: • Qualified consulting pipeline moved from _$118k to $164k_ over the last 10 days. • Two enterprise advisory opportunities are now in procurement review. • The near-term risk is slower legal turnaround on MSA redlines, which could push one April close into May.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -760,83 +768,127 @@
         <x:v>Highlight</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Make the narrative concrete: growth is working, but reliability and enterprise readiness still need disciplined execution.</x:v>
+        <x:v>C09MXSVB2HH: Hyperagent is a good alternative for clients, in advanced talks with RTPL for its implementaiotn on behalf of DB consulting and Advisory</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Leadership/Slack</x:v>
+        <x:v>Slack/GitHub</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Ask</x:v>
+        <x:v>Risk</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
+        <x:v>C09MXSVB2HH: • One client workshop is blocked until the data room access issue is resolved. • Delivery confidence remains high, but the team needs a named owner for exec stakeholder scheduling. • If we do not unblock the security questionnaire by Friday, the healthcare advisory kickoff will slip by at least one week.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Leadership/Slack</x:v>
+        <x:v>Slack/GitHub</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Ask</x:v>
+        <x:v>Risk</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
+        <x:v>Open issue #5: Risk: Live channel quality can overwhelm executive-briefing signal</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>slack</x:v>
+        <x:v>Slack/GitHub</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>implemented</x:v>
+        <x:v>Risk</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Live Slack API adapter for 2 channel(s)</x:v>
+        <x:v>Open issue #4: Future idea: Add client-ready QBR output mode</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>github</x:v>
+        <x:v>Leadership/Slack</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>implemented</x:v>
+        <x:v>Ask</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>Live GitHub API adapter for Laksh-star/codex-workflow-agents</x:v>
+        <x:v>C09MXSVB2HH: • Need approval to pull one additional analytics contractor into the customer-ops workstream for 3 weeks. • Need legal support on the enterprise MSA backlog to protect April revenue timing. • Please confirm whether we want the board narrative to emphasize pipeline quality, delivery readiness, or margin improvement first.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>local-notes</x:v>
+        <x:v>Leadership/Slack</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>implemented</x:v>
+        <x:v>Ask</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>Local document ingestion</x:v>
+        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>kpi-file</x:v>
+        <x:v>Leadership/Slack</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>implemented</x:v>
+        <x:v>Ask</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>Spreadsheet/file ingestion</x:v>
+        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
+        <x:v>slack</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Live Slack API adapter for 1 channel(s)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>github</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Live GitHub API adapter for Laksh-star/codex-workflow-agents</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>local-notes</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Local document ingestion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>kpi-file</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>implemented</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Spreadsheet/file ingestion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
         <x:v>computer-use</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c r="B15" t="str">
         <x:v>stubbed</x:v>
       </x:c>
-      <x:c r="C11" t="str">
+      <x:c r="C15" t="str">
         <x:v>computer-use for UI-only dashboards and internal tools</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Curate final consulting demo inputs and outputs
</commit_message>
<xml_diff>
--- a/outputs/executive-briefing-machine-demo/executive-briefing-demo.xlsx
+++ b/outputs/executive-briefing-machine-demo/executive-briefing-demo.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R611cf8399d664131"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="R52320bc482874aad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="3" r:id="R884a9bf76a484d8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rddc9fe9d88c84728"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Data" sheetId="2" r:id="R1754da551d924a3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Notes" sheetId="3" r:id="Ra6638ff4e5da4af3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -228,7 +228,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R16ff1b2fdd0944b9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R26f9b25478d0431f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -401,7 +401,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" t="str">
-        <x:v>Growth and efficiency improved this month, with reliability still the main watch item.</x:v>
+        <x:v>Revenue quality and operating discipline improved this month, with delivery execution still the main watch item.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -426,10 +426,10 @@
         <x:v>ARR</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>$1688k</x:v>
+        <x:v>$869k</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>+64k vs last month</x:v>
+        <x:v>+67k vs last month</x:v>
       </x:c>
       <x:c r="E5" t="str">
         <x:v>C09MXSVB2HH: • The CEO of the retail client said the weekly advisory cadence is working, but they want tighter decision logs and clearer owner follow-through. • The operations lead asked for a dashboard pack that shows burn, renewal risk, and implementation blockers in one place. • This is a good expansion signal if we package the reporting layer cleanly.</x:v>
@@ -443,16 +443,16 @@
         <x:v>Qualified Pipeline</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>$1335k</x:v>
+        <x:v>$772k</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>+85k vs last month</x:v>
+        <x:v>+84k vs last month</x:v>
       </x:c>
       <x:c r="E6" t="str">
         <x:v>C09MXSVB2HH: • Qualified consulting pipeline moved from _$118k to $164k_ over the last 10 days. • Two enterprise advisory opportunities are now in procurement review. • The near-term risk is slower legal turnaround on MSA redlines, which could push one April close into May.</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>Open issue #5: Risk: Live channel quality can overwhelm executive-briefing signal</x:v>
+        <x:v>Risk #5: Risk: Live channel quality can overwhelm executive-briefing signal</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -460,7 +460,7 @@
         <x:v>Net Burn</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>$226k</x:v>
+        <x:v>$121k</x:v>
       </x:c>
       <x:c r="C7" t="str">
         <x:v>-5k vs last month</x:v>
@@ -468,19 +468,17 @@
       <x:c r="E7" t="str">
         <x:v>C09MXSVB2HH: Hyperagent is a good alternative for clients, in advanced talks with RTPL for its implementaiotn on behalf of DB consulting and Advisory</x:v>
       </x:c>
-      <x:c r="F7" t="str">
-        <x:v>Open issue #4: Future idea: Add client-ready QBR output mode</x:v>
-      </x:c>
+      <x:c r="F7" t="str"/>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" t="str">
         <x:v>NRR</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>114%</x:v>
+        <x:v>111%</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>+1 pts vs last month</x:v>
+        <x:v>+2 pts vs last month</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
@@ -488,10 +486,10 @@
         <x:v>Sev-1 Incidents</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>+1 incident improvement</x:v>
+        <x:v>0 incident improvement</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -518,7 +516,7 @@
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
       <x:c r="A13" t="str">
-        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
+        <x:v>The board narrative should show that Directing Business Consulting Advisory is becoming a repeatable boutique AI advisory business, not a collection of one-off projects.</x:v>
       </x:c>
       <x:c r="B13" t="str">
         <x:v>Product / Engineering</x:v>
@@ -529,7 +527,7 @@
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
       <x:c r="A14" t="str">
-        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
+        <x:v>Emphasize conversion from founder-led consulting into packaged offerings: chief-of-staff systems, GTM operating cadence, and AI-enabled advisory retainers.</x:v>
       </x:c>
       <x:c r="B14" t="str">
         <x:v>Leadership team</x:v>
@@ -597,19 +595,19 @@
         <x:v>Jan 26</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>1420</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="C2" t="n">
-        <x:v>980</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="D2" t="n">
-        <x:v>255</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="E2" t="n">
-        <x:v>109</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="F2" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -617,19 +615,19 @@
         <x:v>Feb 26</x:v>
       </x:c>
       <x:c r="B3" t="n">
-        <x:v>1465</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="C3" t="n">
-        <x:v>1020</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="D3" t="n">
-        <x:v>248</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="E3" t="n">
-        <x:v>110</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="F3" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -637,19 +635,19 @@
         <x:v>Mar 26</x:v>
       </x:c>
       <x:c r="B4" t="n">
-        <x:v>1510</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="C4" t="n">
-        <x:v>1085</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="D4" t="n">
-        <x:v>244</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="E4" t="n">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="F4" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -657,19 +655,19 @@
         <x:v>Apr 26</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:v>1568</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="C5" t="n">
-        <x:v>1175</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="D5" t="n">
-        <x:v>238</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:v>112</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F5" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -677,19 +675,19 @@
         <x:v>May 26</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>1624</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="C6" t="n">
-        <x:v>1250</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="D6" t="n">
-        <x:v>231</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="E6" t="n">
-        <x:v>113</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="F6" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -697,24 +695,24 @@
         <x:v>Jun 26</x:v>
       </x:c>
       <x:c r="B7" t="n">
-        <x:v>1688</x:v>
+        <x:v>869</x:v>
       </x:c>
       <x:c r="C7" t="n">
-        <x:v>1335</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="D7" t="n">
-        <x:v>226</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="E7" t="n">
-        <x:v>114</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="F7" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56fbe2dad6b6428e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c670f6e4baa43e1"/>
 </x:worksheet>
 </file>
 
@@ -790,18 +788,18 @@
         <x:v>Risk</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>Open issue #5: Risk: Live channel quality can overwhelm executive-briefing signal</x:v>
+        <x:v>Risk #5: Risk: Live channel quality can overwhelm executive-briefing signal</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Slack/GitHub</x:v>
+        <x:v>Leadership/Slack</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Risk</x:v>
+        <x:v>Ask</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Open issue #4: Future idea: Add client-ready QBR output mode</x:v>
+        <x:v>C09MXSVB2HH: • Need approval to pull one additional analytics contractor into the customer-ops workstream for 3 weeks. • Need legal support on the enterprise MSA backlog to protect April revenue timing. • Please confirm whether we want the board narrative to emphasize pipeline quality, delivery readiness, or margin improvement first.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -812,7 +810,7 @@
         <x:v>Ask</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>C09MXSVB2HH: • Need approval to pull one additional analytics contractor into the customer-ops workstream for 3 weeks. • Need legal support on the enterprise MSA backlog to protect April revenue timing. • Please confirm whether we want the board narrative to emphasize pipeline quality, delivery readiness, or margin improvement first.</x:v>
+        <x:v>The board narrative should show that Directing Business Consulting Advisory is becoming a repeatable boutique AI advisory business, not a collection of one-off projects.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -823,72 +821,61 @@
         <x:v>Ask</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>The board will care most about whether enterprise pipeline supports the Q3 revenue target.</x:v>
+        <x:v>Emphasize conversion from founder-led consulting into packaged offerings: chief-of-staff systems, GTM operating cadence, and AI-enabled advisory retainers.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>Leadership/Slack</x:v>
+        <x:v>slack</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>Ask</x:v>
+        <x:v>implemented</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>Keep net burn under $230k while continuing to invest in product reliability.</x:v>
+        <x:v>Live Slack API adapter for 1 channel(s)</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>slack</x:v>
+        <x:v>github</x:v>
       </x:c>
       <x:c r="B11" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>Live Slack API adapter for 1 channel(s)</x:v>
+        <x:v>Live GitHub API adapter for Laksh-star/codex-workflow-agents</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>github</x:v>
+        <x:v>local-notes</x:v>
       </x:c>
       <x:c r="B12" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Live GitHub API adapter for Laksh-star/codex-workflow-agents</x:v>
+        <x:v>Local document ingestion</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>local-notes</x:v>
+        <x:v>kpi-file</x:v>
       </x:c>
       <x:c r="B13" t="str">
         <x:v>implemented</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>Local document ingestion</x:v>
+        <x:v>Spreadsheet/file ingestion</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>kpi-file</x:v>
+        <x:v>computer-use</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>implemented</x:v>
+        <x:v>stubbed</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>Spreadsheet/file ingestion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>computer-use</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>stubbed</x:v>
-      </x:c>
-      <x:c r="C15" t="str">
         <x:v>computer-use for UI-only dashboards and internal tools</x:v>
       </x:c>
     </x:row>

</xml_diff>